<commit_message>
EAINT-12341: order runs by business-type priority (QA request)
Sdn Bhd / Bhd > Sole Proprietorship / Partnership > LLP > Business Trading
(Sabah) > Business Trading (Sarawak). Runs renumbered so CH1..CH8 is the
execution order; the main run (extra checks CH1-20, CH1-21) is now the
Sdn Bhd 4-director run. Workbook, eSim setup sheet, robot, guide, prompts
and status follow the same order. The robot now refuses a company whose
TIN prefix does not fit the run's business type, before anything is
written.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_015cZiRisoA6SpsRKpMC9zuJ
</commit_message>
<xml_diff>
--- a/EAINT-12341/cr/EAINT-12341/02-plan/EAINT-12341_eSim_Setup.xlsx
+++ b/EAINT-12341/cr/EAINT-12341/02-plan/EAINT-12341_eSim_Setup.xlsx
@@ -11,10 +11,10 @@
     <sheet name="1 Companies" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="CH1" sheetId="3" state="visible" r:id="rId3"/>
     <sheet name="CH2" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="CH6" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="CH3" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="CH8" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet name="CH4" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="CH3" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="CH4" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="CH5" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="CH6" sheetId="8" state="visible" r:id="rId8"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -606,7 +606,7 @@
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>Business Trading (CH5 Sabah, CH7 Sarawak) has no eSim setup — fill only its TIN in tab 1.</t>
+          <t>Business Trading (CH7 Sabah, CH8 Sarawak) has no eSim setup — fill only its TIN in tab 1.</t>
         </is>
       </c>
     </row>
@@ -718,12 +718,12 @@
       </c>
       <c r="C4" s="6" t="inlineStr">
         <is>
-          <t>Sole Prop / Partnership</t>
+          <t>Sdn Bhd / Bhd</t>
         </is>
       </c>
       <c r="D4" s="6" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>C</t>
         </is>
       </c>
       <c r="E4" s="6" t="inlineStr">
@@ -737,7 +737,7 @@
       <c r="I4" s="7" t="n"/>
       <c r="J4" s="6" t="inlineStr">
         <is>
-          <t>Main test, run first</t>
+          <t>MAIN TEST — run first</t>
         </is>
       </c>
       <c r="K4" s="8">
@@ -760,24 +760,28 @@
       </c>
       <c r="C5" s="6" t="inlineStr">
         <is>
-          <t>Sole Prop / Partnership</t>
+          <t>Sdn Bhd / Bhd</t>
         </is>
       </c>
       <c r="D5" s="6" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>C</t>
         </is>
       </c>
       <c r="E5" s="6" t="inlineStr">
         <is>
-          <t>5 Malaysian</t>
+          <t>2 Malaysian + 1 foreigner</t>
         </is>
       </c>
       <c r="F5" s="7" t="n"/>
       <c r="G5" s="7" t="n"/>
       <c r="H5" s="7" t="n"/>
       <c r="I5" s="7" t="n"/>
-      <c r="J5" s="6" t="inlineStr"/>
+      <c r="J5" s="6" t="inlineStr">
+        <is>
+          <t>Has 1 foreign director</t>
+        </is>
+      </c>
       <c r="K5" s="8">
         <f>IF(F5="","",IF(AND(LEN(F5)&gt;2,MID(F5,LEN(F5)-1,1)="-",ISERROR(VALUE(RIGHT(F5,1)))),LEFT(F5,LEN(F5)-2),F5))</f>
         <v/>
@@ -793,7 +797,7 @@
       </c>
       <c r="B6" s="6" t="inlineStr">
         <is>
-          <t>CH6</t>
+          <t>CH3</t>
         </is>
       </c>
       <c r="C6" s="6" t="inlineStr">
@@ -803,7 +807,7 @@
       </c>
       <c r="D6" s="6" t="inlineStr">
         <is>
-          <t>D (or IG)</t>
+          <t>D</t>
         </is>
       </c>
       <c r="E6" s="6" t="inlineStr">
@@ -815,11 +819,7 @@
       <c r="G6" s="7" t="n"/>
       <c r="H6" s="7" t="n"/>
       <c r="I6" s="7" t="n"/>
-      <c r="J6" s="6" t="inlineStr">
-        <is>
-          <t>Stops at Submitted</t>
-        </is>
-      </c>
+      <c r="J6" s="6" t="inlineStr"/>
       <c r="K6" s="8">
         <f>IF(F6="","",IF(AND(LEN(F6)&gt;2,MID(F6,LEN(F6)-1,1)="-",ISERROR(VALUE(RIGHT(F6,1)))),LEFT(F6,LEN(F6)-2),F6))</f>
         <v/>
@@ -835,33 +835,29 @@
       </c>
       <c r="B7" s="6" t="inlineStr">
         <is>
-          <t>CH3</t>
+          <t>CH4</t>
         </is>
       </c>
       <c r="C7" s="6" t="inlineStr">
         <is>
-          <t>Sdn Bhd / Bhd</t>
+          <t>Sole Prop / Partnership</t>
         </is>
       </c>
       <c r="D7" s="6" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>D</t>
         </is>
       </c>
       <c r="E7" s="6" t="inlineStr">
         <is>
-          <t>2 Malaysian + 1 foreigner</t>
+          <t>5 Malaysian</t>
         </is>
       </c>
       <c r="F7" s="7" t="n"/>
       <c r="G7" s="7" t="n"/>
       <c r="H7" s="7" t="n"/>
       <c r="I7" s="7" t="n"/>
-      <c r="J7" s="6" t="inlineStr">
-        <is>
-          <t>Has 1 foreign director</t>
-        </is>
-      </c>
+      <c r="J7" s="6" t="inlineStr"/>
       <c r="K7" s="8">
         <f>IF(F7="","",IF(AND(LEN(F7)&gt;2,MID(F7,LEN(F7)-1,1)="-",ISERROR(VALUE(RIGHT(F7,1)))),LEFT(F7,LEN(F7)-2),F7))</f>
         <v/>
@@ -877,17 +873,17 @@
       </c>
       <c r="B8" s="6" t="inlineStr">
         <is>
-          <t>CH8</t>
+          <t>CH5</t>
         </is>
       </c>
       <c r="C8" s="6" t="inlineStr">
         <is>
-          <t>Sdn Bhd / Bhd</t>
+          <t>Sole Prop / Partnership</t>
         </is>
       </c>
       <c r="D8" s="6" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>D (or IG)</t>
         </is>
       </c>
       <c r="E8" s="6" t="inlineStr">
@@ -901,7 +897,7 @@
       <c r="I8" s="7" t="n"/>
       <c r="J8" s="6" t="inlineStr">
         <is>
-          <t>Normal Sdn Bhd case</t>
+          <t>Stops at Submitted</t>
         </is>
       </c>
       <c r="K8" s="8">
@@ -919,7 +915,7 @@
       </c>
       <c r="B9" s="6" t="inlineStr">
         <is>
-          <t>CH4</t>
+          <t>CH6</t>
         </is>
       </c>
       <c r="C9" s="6" t="inlineStr">
@@ -961,7 +957,7 @@
       </c>
       <c r="B10" s="6" t="inlineStr">
         <is>
-          <t>CH5</t>
+          <t>CH7</t>
         </is>
       </c>
       <c r="C10" s="6" t="inlineStr">
@@ -1003,7 +999,7 @@
       </c>
       <c r="B11" s="6" t="inlineStr">
         <is>
-          <t>CH7</t>
+          <t>CH8</t>
         </is>
       </c>
       <c r="C11" s="6" t="inlineStr">
@@ -1050,12 +1046,12 @@
       </c>
       <c r="C12" s="6" t="inlineStr">
         <is>
-          <t>Sole Prop / Partnership</t>
+          <t>Sdn Bhd / Bhd</t>
         </is>
       </c>
       <c r="D12" s="6" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>C</t>
         </is>
       </c>
       <c r="E12" s="6" t="inlineStr">
@@ -1134,12 +1130,12 @@
       </c>
       <c r="C14" s="6" t="inlineStr">
         <is>
-          <t>Sdn Bhd / Bhd</t>
+          <t>Sole Prop / Partnership</t>
         </is>
       </c>
       <c r="D14" s="6" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>D</t>
         </is>
       </c>
       <c r="E14" s="6" t="inlineStr">
@@ -1289,14 +1285,14 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>CH1 — Sole Prop / Partnership — Main test, run first</t>
+          <t>CH1 — Sdn Bhd / Bhd — MAIN TEST — run first</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Company name the robot types: QA 12341 CH1 ENTERPRISE</t>
+          <t>Company name the robot types: QA 12341 CH1 SDN BHD</t>
         </is>
       </c>
     </row>
@@ -1393,7 +1389,7 @@
       </c>
       <c r="B10" s="6" t="inlineStr">
         <is>
-          <t>QA 12341 CH1 ENTERPRISE</t>
+          <t>QA 12341 CH1 SDN BHD</t>
         </is>
       </c>
       <c r="C10" s="6" t="inlineStr">
@@ -1418,7 +1414,7 @@
     <row r="13">
       <c r="A13" s="10" t="inlineStr">
         <is>
-          <t>Part B — screen 'Ssm Rob Submission Resp' (edit a record, then Save)</t>
+          <t>Part B — screen 'Ssm Roc Submission Resp' (edit a record, then Save)</t>
         </is>
       </c>
     </row>
@@ -1508,7 +1504,7 @@
       </c>
       <c r="B19" s="6" t="inlineStr">
         <is>
-          <t>QA 12341 CH1 ENTERPRISE</t>
+          <t>QA 12341 CH1 SDN BHD</t>
         </is>
       </c>
       <c r="C19" s="6" t="inlineStr"/>
@@ -1533,7 +1529,7 @@
     <row r="22">
       <c r="A22" s="10" t="inlineStr">
         <is>
-          <t>Part B — text box 'Business Info': change ONLY these tags</t>
+          <t>Part B — text box 'Page 1': change ONLY these tags</t>
         </is>
       </c>
     </row>
@@ -1557,11 +1553,11 @@
     <row r="24">
       <c r="A24" s="6" t="inlineStr">
         <is>
-          <t>&lt;BUSINESS_REF_NO&gt;</t>
+          <t>&lt;REF_NO&gt;</t>
         </is>
       </c>
       <c r="B24" s="8">
-        <f>"&lt;BUSINESS_REF_NO&gt;"&amp;IF('1 Companies'!F4="","(fill tab 1 first)",'1 Companies'!F4)&amp;"&lt;/BUSINESS_REF_NO&gt;"</f>
+        <f>"&lt;REF_NO&gt;"&amp;IF('1 Companies'!F4="","(fill tab 1 first)",'1 Companies'!F4)&amp;"&lt;/REF_NO&gt;"</f>
         <v/>
       </c>
       <c r="C24" s="6" t="inlineStr">
@@ -1585,12 +1581,12 @@
     <row r="26">
       <c r="A26" s="6" t="inlineStr">
         <is>
-          <t>&lt;ROB_STATUS&gt;</t>
+          <t>&lt;ROC_STATUS&gt;</t>
         </is>
       </c>
       <c r="B26" s="6" t="inlineStr">
         <is>
-          <t>&lt;ROB_STATUS&gt;ACTIVE&lt;/ROB_STATUS&gt;</t>
+          <t>&lt;ROC_STATUS&gt;EXISTING&lt;/ROC_STATUS&gt;</t>
         </is>
       </c>
       <c r="C26" s="6" t="inlineStr"/>
@@ -1598,7 +1594,7 @@
     <row r="28">
       <c r="A28" s="10" t="inlineStr">
         <is>
-          <t>Part B — text box 'Current Owner Info': exactly 4 owner blocks</t>
+          <t>Part B — text box 'Page 3': exactly 4 director blocks (designation DIRECTOR)</t>
         </is>
       </c>
     </row>
@@ -1639,12 +1635,12 @@
     <row r="31">
       <c r="A31" s="6" t="inlineStr">
         <is>
-          <t>Person A — &lt;IC_NEW&gt; (no dashes)</t>
+          <t>Person A — &lt;IC&gt; (with dashes)</t>
         </is>
       </c>
       <c r="B31" s="6" t="inlineStr">
         <is>
-          <t>690501137631</t>
+          <t>690501-13-7631</t>
         </is>
       </c>
       <c r="C31" s="6" t="inlineStr"/>
@@ -1669,12 +1665,12 @@
     <row r="33">
       <c r="A33" s="6" t="inlineStr">
         <is>
-          <t>Person B — &lt;IC_NEW&gt; (no dashes)</t>
+          <t>Person B — &lt;IC&gt; (with dashes)</t>
         </is>
       </c>
       <c r="B33" s="6" t="inlineStr">
         <is>
-          <t>690502137632</t>
+          <t>690502-13-7632</t>
         </is>
       </c>
       <c r="C33" s="6" t="inlineStr"/>
@@ -1699,12 +1695,12 @@
     <row r="35">
       <c r="A35" s="6" t="inlineStr">
         <is>
-          <t>Person C — &lt;IC_NEW&gt; (no dashes)</t>
+          <t>Person C — &lt;IC&gt; (with dashes)</t>
         </is>
       </c>
       <c r="B35" s="6" t="inlineStr">
         <is>
-          <t>690503137633</t>
+          <t>690503-13-7633</t>
         </is>
       </c>
       <c r="C35" s="6" t="inlineStr"/>
@@ -1729,12 +1725,12 @@
     <row r="37">
       <c r="A37" s="6" t="inlineStr">
         <is>
-          <t>Person D — &lt;IC_NEW&gt; (no dashes)</t>
+          <t>Person D — &lt;IC&gt; (with dashes)</t>
         </is>
       </c>
       <c r="B37" s="6" t="inlineStr">
         <is>
-          <t>690504137634</t>
+          <t>690504-13-7634</t>
         </is>
       </c>
       <c r="C37" s="6" t="inlineStr"/>
@@ -1763,7 +1759,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C41"/>
+  <dimension ref="A1:C37"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -1774,14 +1770,14 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>CH2 — Sole Prop / Partnership — set up just before running ch2</t>
+          <t>CH2 — Sdn Bhd / Bhd — Has 1 foreign director</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Company name the robot types: QA 12341 CH2 ENTERPRISE</t>
+          <t>Company name the robot types: QA 12341 CH2 SDN BHD</t>
         </is>
       </c>
     </row>
@@ -1878,7 +1874,7 @@
       </c>
       <c r="B10" s="6" t="inlineStr">
         <is>
-          <t>QA 12341 CH2 ENTERPRISE</t>
+          <t>QA 12341 CH2 SDN BHD</t>
         </is>
       </c>
       <c r="C10" s="6" t="inlineStr">
@@ -1903,7 +1899,7 @@
     <row r="13">
       <c r="A13" s="10" t="inlineStr">
         <is>
-          <t>Part B — screen 'Ssm Rob Submission Resp' (edit a record, then Save)</t>
+          <t>Part B — screen 'Ssm Roc Submission Resp' (edit a record, then Save)</t>
         </is>
       </c>
     </row>
@@ -1993,7 +1989,7 @@
       </c>
       <c r="B19" s="6" t="inlineStr">
         <is>
-          <t>QA 12341 CH2 ENTERPRISE</t>
+          <t>QA 12341 CH2 SDN BHD</t>
         </is>
       </c>
       <c r="C19" s="6" t="inlineStr"/>
@@ -2018,7 +2014,7 @@
     <row r="22">
       <c r="A22" s="10" t="inlineStr">
         <is>
-          <t>Part B — text box 'Business Info': change ONLY these tags</t>
+          <t>Part B — text box 'Page 1': change ONLY these tags</t>
         </is>
       </c>
     </row>
@@ -2042,11 +2038,11 @@
     <row r="24">
       <c r="A24" s="6" t="inlineStr">
         <is>
-          <t>&lt;BUSINESS_REF_NO&gt;</t>
+          <t>&lt;REF_NO&gt;</t>
         </is>
       </c>
       <c r="B24" s="8">
-        <f>"&lt;BUSINESS_REF_NO&gt;"&amp;IF('1 Companies'!F5="","(fill tab 1 first)",'1 Companies'!F5)&amp;"&lt;/BUSINESS_REF_NO&gt;"</f>
+        <f>"&lt;REF_NO&gt;"&amp;IF('1 Companies'!F5="","(fill tab 1 first)",'1 Companies'!F5)&amp;"&lt;/REF_NO&gt;"</f>
         <v/>
       </c>
       <c r="C24" s="6" t="inlineStr">
@@ -2070,12 +2066,12 @@
     <row r="26">
       <c r="A26" s="6" t="inlineStr">
         <is>
-          <t>&lt;ROB_STATUS&gt;</t>
+          <t>&lt;ROC_STATUS&gt;</t>
         </is>
       </c>
       <c r="B26" s="6" t="inlineStr">
         <is>
-          <t>&lt;ROB_STATUS&gt;ACTIVE&lt;/ROB_STATUS&gt;</t>
+          <t>&lt;ROC_STATUS&gt;EXISTING&lt;/ROC_STATUS&gt;</t>
         </is>
       </c>
       <c r="C26" s="6" t="inlineStr"/>
@@ -2083,7 +2079,7 @@
     <row r="28">
       <c r="A28" s="10" t="inlineStr">
         <is>
-          <t>Part B — text box 'Current Owner Info': exactly 5 owner blocks</t>
+          <t>Part B — text box 'Page 3': exactly 3 director blocks (designation DIRECTOR)</t>
         </is>
       </c>
     </row>
@@ -2124,12 +2120,12 @@
     <row r="31">
       <c r="A31" s="6" t="inlineStr">
         <is>
-          <t>Person A — &lt;IC_NEW&gt; (no dashes)</t>
+          <t>Person A — &lt;IC&gt; (with dashes)</t>
         </is>
       </c>
       <c r="B31" s="6" t="inlineStr">
         <is>
-          <t>690501137631</t>
+          <t>690501-13-7631</t>
         </is>
       </c>
       <c r="C31" s="6" t="inlineStr"/>
@@ -2154,12 +2150,12 @@
     <row r="33">
       <c r="A33" s="6" t="inlineStr">
         <is>
-          <t>Person B — &lt;IC_NEW&gt; (no dashes)</t>
+          <t>Person B — &lt;IC&gt; (with dashes)</t>
         </is>
       </c>
       <c r="B33" s="6" t="inlineStr">
         <is>
-          <t>690502137632</t>
+          <t>690502-13-7632</t>
         </is>
       </c>
       <c r="C33" s="6" t="inlineStr"/>
@@ -2177,85 +2173,25 @@
       </c>
       <c r="C34" s="6" t="inlineStr">
         <is>
-          <t>Malaysian</t>
+          <t>Foreign director — ID format to confirm</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="6" t="inlineStr">
         <is>
-          <t>Person C — &lt;IC_NEW&gt; (no dashes)</t>
+          <t>Person C — &lt;IC&gt; (with dashes)</t>
         </is>
       </c>
       <c r="B35" s="6" t="inlineStr">
         <is>
-          <t>690503137633</t>
+          <t>A12345672</t>
         </is>
       </c>
       <c r="C35" s="6" t="inlineStr"/>
     </row>
-    <row r="36">
-      <c r="A36" s="6" t="inlineStr">
-        <is>
-          <t>Person D — name</t>
-        </is>
-      </c>
-      <c r="B36" s="6" t="inlineStr">
-        <is>
-          <t>QA DIRECTOR D</t>
-        </is>
-      </c>
-      <c r="C36" s="6" t="inlineStr">
-        <is>
-          <t>Malaysian</t>
-        </is>
-      </c>
-    </row>
     <row r="37">
-      <c r="A37" s="6" t="inlineStr">
-        <is>
-          <t>Person D — &lt;IC_NEW&gt; (no dashes)</t>
-        </is>
-      </c>
-      <c r="B37" s="6" t="inlineStr">
-        <is>
-          <t>690504137634</t>
-        </is>
-      </c>
-      <c r="C37" s="6" t="inlineStr"/>
-    </row>
-    <row r="38">
-      <c r="A38" s="6" t="inlineStr">
-        <is>
-          <t>Person E — name</t>
-        </is>
-      </c>
-      <c r="B38" s="6" t="inlineStr">
-        <is>
-          <t>QA DIRECTOR E</t>
-        </is>
-      </c>
-      <c r="C38" s="6" t="inlineStr">
-        <is>
-          <t>Malaysian</t>
-        </is>
-      </c>
-    </row>
-    <row r="39">
-      <c r="A39" s="6" t="inlineStr">
-        <is>
-          <t>Person E — &lt;IC_NEW&gt; (no dashes)</t>
-        </is>
-      </c>
-      <c r="B39" s="6" t="inlineStr">
-        <is>
-          <t>690505137635</t>
-        </is>
-      </c>
-      <c r="C39" s="6" t="inlineStr"/>
-    </row>
-    <row r="41">
-      <c r="A41" s="3" t="inlineStr">
+      <c r="A37" s="3" t="inlineStr">
         <is>
           <t>Then: Save, tell QA support 'eSim ready', and run the robot.</t>
         </is>
@@ -2289,14 +2225,14 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>CH6 — Sole Prop / Partnership — Stops at Submitted</t>
+          <t>CH3 — Sole Prop / Partnership — set up just before running ch3</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Company name the robot types: QA 12341 CH6 ENTERPRISE</t>
+          <t>Company name the robot types: QA 12341 CH3 ENTERPRISE</t>
         </is>
       </c>
     </row>
@@ -2393,7 +2329,7 @@
       </c>
       <c r="B10" s="6" t="inlineStr">
         <is>
-          <t>QA 12341 CH6 ENTERPRISE</t>
+          <t>QA 12341 CH3 ENTERPRISE</t>
         </is>
       </c>
       <c r="C10" s="6" t="inlineStr">
@@ -2508,7 +2444,7 @@
       </c>
       <c r="B19" s="6" t="inlineStr">
         <is>
-          <t>QA 12341 CH6 ENTERPRISE</t>
+          <t>QA 12341 CH3 ENTERPRISE</t>
         </is>
       </c>
       <c r="C19" s="6" t="inlineStr"/>
@@ -2763,7 +2699,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C37"/>
+  <dimension ref="A1:C41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -2774,14 +2710,14 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>CH3 — Sdn Bhd / Bhd — Has 1 foreign director</t>
+          <t>CH4 — Sole Prop / Partnership — set up just before running ch4</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Company name the robot types: QA 12341 CH3 SDN BHD</t>
+          <t>Company name the robot types: QA 12341 CH4 ENTERPRISE</t>
         </is>
       </c>
     </row>
@@ -2878,7 +2814,7 @@
       </c>
       <c r="B10" s="6" t="inlineStr">
         <is>
-          <t>QA 12341 CH3 SDN BHD</t>
+          <t>QA 12341 CH4 ENTERPRISE</t>
         </is>
       </c>
       <c r="C10" s="6" t="inlineStr">
@@ -2903,7 +2839,7 @@
     <row r="13">
       <c r="A13" s="10" t="inlineStr">
         <is>
-          <t>Part B — screen 'Ssm Roc Submission Resp' (edit a record, then Save)</t>
+          <t>Part B — screen 'Ssm Rob Submission Resp' (edit a record, then Save)</t>
         </is>
       </c>
     </row>
@@ -2993,7 +2929,7 @@
       </c>
       <c r="B19" s="6" t="inlineStr">
         <is>
-          <t>QA 12341 CH3 SDN BHD</t>
+          <t>QA 12341 CH4 ENTERPRISE</t>
         </is>
       </c>
       <c r="C19" s="6" t="inlineStr"/>
@@ -3018,7 +2954,7 @@
     <row r="22">
       <c r="A22" s="10" t="inlineStr">
         <is>
-          <t>Part B — text box 'Page 1': change ONLY these tags</t>
+          <t>Part B — text box 'Business Info': change ONLY these tags</t>
         </is>
       </c>
     </row>
@@ -3042,11 +2978,11 @@
     <row r="24">
       <c r="A24" s="6" t="inlineStr">
         <is>
-          <t>&lt;REF_NO&gt;</t>
+          <t>&lt;BUSINESS_REF_NO&gt;</t>
         </is>
       </c>
       <c r="B24" s="8">
-        <f>"&lt;REF_NO&gt;"&amp;IF('1 Companies'!F7="","(fill tab 1 first)",'1 Companies'!F7)&amp;"&lt;/REF_NO&gt;"</f>
+        <f>"&lt;BUSINESS_REF_NO&gt;"&amp;IF('1 Companies'!F7="","(fill tab 1 first)",'1 Companies'!F7)&amp;"&lt;/BUSINESS_REF_NO&gt;"</f>
         <v/>
       </c>
       <c r="C24" s="6" t="inlineStr">
@@ -3070,12 +3006,12 @@
     <row r="26">
       <c r="A26" s="6" t="inlineStr">
         <is>
-          <t>&lt;ROC_STATUS&gt;</t>
+          <t>&lt;ROB_STATUS&gt;</t>
         </is>
       </c>
       <c r="B26" s="6" t="inlineStr">
         <is>
-          <t>&lt;ROC_STATUS&gt;EXISTING&lt;/ROC_STATUS&gt;</t>
+          <t>&lt;ROB_STATUS&gt;ACTIVE&lt;/ROB_STATUS&gt;</t>
         </is>
       </c>
       <c r="C26" s="6" t="inlineStr"/>
@@ -3083,7 +3019,7 @@
     <row r="28">
       <c r="A28" s="10" t="inlineStr">
         <is>
-          <t>Part B — text box 'Page 3': exactly 3 director blocks (designation DIRECTOR)</t>
+          <t>Part B — text box 'Current Owner Info': exactly 5 owner blocks</t>
         </is>
       </c>
     </row>
@@ -3124,12 +3060,12 @@
     <row r="31">
       <c r="A31" s="6" t="inlineStr">
         <is>
-          <t>Person A — &lt;IC&gt; (with dashes)</t>
+          <t>Person A — &lt;IC_NEW&gt; (no dashes)</t>
         </is>
       </c>
       <c r="B31" s="6" t="inlineStr">
         <is>
-          <t>690501-13-7631</t>
+          <t>690501137631</t>
         </is>
       </c>
       <c r="C31" s="6" t="inlineStr"/>
@@ -3154,12 +3090,12 @@
     <row r="33">
       <c r="A33" s="6" t="inlineStr">
         <is>
-          <t>Person B — &lt;IC&gt; (with dashes)</t>
+          <t>Person B — &lt;IC_NEW&gt; (no dashes)</t>
         </is>
       </c>
       <c r="B33" s="6" t="inlineStr">
         <is>
-          <t>690502-13-7632</t>
+          <t>690502137632</t>
         </is>
       </c>
       <c r="C33" s="6" t="inlineStr"/>
@@ -3177,25 +3113,85 @@
       </c>
       <c r="C34" s="6" t="inlineStr">
         <is>
-          <t>Foreign director — ID format to confirm</t>
+          <t>Malaysian</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="6" t="inlineStr">
         <is>
-          <t>Person C — &lt;IC&gt; (with dashes)</t>
+          <t>Person C — &lt;IC_NEW&gt; (no dashes)</t>
         </is>
       </c>
       <c r="B35" s="6" t="inlineStr">
         <is>
-          <t>A12345672</t>
+          <t>690503137633</t>
         </is>
       </c>
       <c r="C35" s="6" t="inlineStr"/>
     </row>
+    <row r="36">
+      <c r="A36" s="6" t="inlineStr">
+        <is>
+          <t>Person D — name</t>
+        </is>
+      </c>
+      <c r="B36" s="6" t="inlineStr">
+        <is>
+          <t>QA DIRECTOR D</t>
+        </is>
+      </c>
+      <c r="C36" s="6" t="inlineStr">
+        <is>
+          <t>Malaysian</t>
+        </is>
+      </c>
+    </row>
     <row r="37">
-      <c r="A37" s="3" t="inlineStr">
+      <c r="A37" s="6" t="inlineStr">
+        <is>
+          <t>Person D — &lt;IC_NEW&gt; (no dashes)</t>
+        </is>
+      </c>
+      <c r="B37" s="6" t="inlineStr">
+        <is>
+          <t>690504137634</t>
+        </is>
+      </c>
+      <c r="C37" s="6" t="inlineStr"/>
+    </row>
+    <row r="38">
+      <c r="A38" s="6" t="inlineStr">
+        <is>
+          <t>Person E — name</t>
+        </is>
+      </c>
+      <c r="B38" s="6" t="inlineStr">
+        <is>
+          <t>QA DIRECTOR E</t>
+        </is>
+      </c>
+      <c r="C38" s="6" t="inlineStr">
+        <is>
+          <t>Malaysian</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="6" t="inlineStr">
+        <is>
+          <t>Person E — &lt;IC_NEW&gt; (no dashes)</t>
+        </is>
+      </c>
+      <c r="B39" s="6" t="inlineStr">
+        <is>
+          <t>690505137635</t>
+        </is>
+      </c>
+      <c r="C39" s="6" t="inlineStr"/>
+    </row>
+    <row r="41">
+      <c r="A41" s="3" t="inlineStr">
         <is>
           <t>Then: Save, tell QA support 'eSim ready', and run the robot.</t>
         </is>
@@ -3229,14 +3225,14 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>CH8 — Sdn Bhd / Bhd — Normal Sdn Bhd case</t>
+          <t>CH5 — Sole Prop / Partnership — Stops at Submitted</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Company name the robot types: QA 12341 CH8 SDN BHD</t>
+          <t>Company name the robot types: QA 12341 CH5 ENTERPRISE</t>
         </is>
       </c>
     </row>
@@ -3333,7 +3329,7 @@
       </c>
       <c r="B10" s="6" t="inlineStr">
         <is>
-          <t>QA 12341 CH8 SDN BHD</t>
+          <t>QA 12341 CH5 ENTERPRISE</t>
         </is>
       </c>
       <c r="C10" s="6" t="inlineStr">
@@ -3358,7 +3354,7 @@
     <row r="13">
       <c r="A13" s="10" t="inlineStr">
         <is>
-          <t>Part B — screen 'Ssm Roc Submission Resp' (edit a record, then Save)</t>
+          <t>Part B — screen 'Ssm Rob Submission Resp' (edit a record, then Save)</t>
         </is>
       </c>
     </row>
@@ -3448,7 +3444,7 @@
       </c>
       <c r="B19" s="6" t="inlineStr">
         <is>
-          <t>QA 12341 CH8 SDN BHD</t>
+          <t>QA 12341 CH5 ENTERPRISE</t>
         </is>
       </c>
       <c r="C19" s="6" t="inlineStr"/>
@@ -3473,7 +3469,7 @@
     <row r="22">
       <c r="A22" s="10" t="inlineStr">
         <is>
-          <t>Part B — text box 'Page 1': change ONLY these tags</t>
+          <t>Part B — text box 'Business Info': change ONLY these tags</t>
         </is>
       </c>
     </row>
@@ -3497,11 +3493,11 @@
     <row r="24">
       <c r="A24" s="6" t="inlineStr">
         <is>
-          <t>&lt;REF_NO&gt;</t>
+          <t>&lt;BUSINESS_REF_NO&gt;</t>
         </is>
       </c>
       <c r="B24" s="8">
-        <f>"&lt;REF_NO&gt;"&amp;IF('1 Companies'!F8="","(fill tab 1 first)",'1 Companies'!F8)&amp;"&lt;/REF_NO&gt;"</f>
+        <f>"&lt;BUSINESS_REF_NO&gt;"&amp;IF('1 Companies'!F8="","(fill tab 1 first)",'1 Companies'!F8)&amp;"&lt;/BUSINESS_REF_NO&gt;"</f>
         <v/>
       </c>
       <c r="C24" s="6" t="inlineStr">
@@ -3525,12 +3521,12 @@
     <row r="26">
       <c r="A26" s="6" t="inlineStr">
         <is>
-          <t>&lt;ROC_STATUS&gt;</t>
+          <t>&lt;ROB_STATUS&gt;</t>
         </is>
       </c>
       <c r="B26" s="6" t="inlineStr">
         <is>
-          <t>&lt;ROC_STATUS&gt;EXISTING&lt;/ROC_STATUS&gt;</t>
+          <t>&lt;ROB_STATUS&gt;ACTIVE&lt;/ROB_STATUS&gt;</t>
         </is>
       </c>
       <c r="C26" s="6" t="inlineStr"/>
@@ -3538,7 +3534,7 @@
     <row r="28">
       <c r="A28" s="10" t="inlineStr">
         <is>
-          <t>Part B — text box 'Page 3': exactly 4 director blocks (designation DIRECTOR)</t>
+          <t>Part B — text box 'Current Owner Info': exactly 4 owner blocks</t>
         </is>
       </c>
     </row>
@@ -3579,12 +3575,12 @@
     <row r="31">
       <c r="A31" s="6" t="inlineStr">
         <is>
-          <t>Person A — &lt;IC&gt; (with dashes)</t>
+          <t>Person A — &lt;IC_NEW&gt; (no dashes)</t>
         </is>
       </c>
       <c r="B31" s="6" t="inlineStr">
         <is>
-          <t>690501-13-7631</t>
+          <t>690501137631</t>
         </is>
       </c>
       <c r="C31" s="6" t="inlineStr"/>
@@ -3609,12 +3605,12 @@
     <row r="33">
       <c r="A33" s="6" t="inlineStr">
         <is>
-          <t>Person B — &lt;IC&gt; (with dashes)</t>
+          <t>Person B — &lt;IC_NEW&gt; (no dashes)</t>
         </is>
       </c>
       <c r="B33" s="6" t="inlineStr">
         <is>
-          <t>690502-13-7632</t>
+          <t>690502137632</t>
         </is>
       </c>
       <c r="C33" s="6" t="inlineStr"/>
@@ -3639,12 +3635,12 @@
     <row r="35">
       <c r="A35" s="6" t="inlineStr">
         <is>
-          <t>Person C — &lt;IC&gt; (with dashes)</t>
+          <t>Person C — &lt;IC_NEW&gt; (no dashes)</t>
         </is>
       </c>
       <c r="B35" s="6" t="inlineStr">
         <is>
-          <t>690503-13-7633</t>
+          <t>690503137633</t>
         </is>
       </c>
       <c r="C35" s="6" t="inlineStr"/>
@@ -3669,12 +3665,12 @@
     <row r="37">
       <c r="A37" s="6" t="inlineStr">
         <is>
-          <t>Person D — &lt;IC&gt; (with dashes)</t>
+          <t>Person D — &lt;IC_NEW&gt; (no dashes)</t>
         </is>
       </c>
       <c r="B37" s="6" t="inlineStr">
         <is>
-          <t>690504-13-7634</t>
+          <t>690504137634</t>
         </is>
       </c>
       <c r="C37" s="6" t="inlineStr"/>
@@ -3714,14 +3710,14 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>CH4 — LLP — Check LLP0035174-LGN first</t>
+          <t>CH6 — LLP — Check LLP0035174-LGN first</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Company name the robot types: QA 12341 CH4 PLT</t>
+          <t>Company name the robot types: QA 12341 CH6 PLT</t>
         </is>
       </c>
     </row>
@@ -3818,7 +3814,7 @@
       </c>
       <c r="B10" s="6" t="inlineStr">
         <is>
-          <t>QA 12341 CH4 PLT</t>
+          <t>QA 12341 CH6 PLT</t>
         </is>
       </c>
       <c r="C10" s="6" t="inlineStr">
@@ -3933,7 +3929,7 @@
       </c>
       <c r="B19" s="6" t="inlineStr">
         <is>
-          <t>QA 12341 CH4 PLT</t>
+          <t>QA 12341 CH6 PLT</t>
         </is>
       </c>
       <c r="C19" s="6" t="inlineStr"/>

</xml_diff>

<commit_message>
EAINT-12341: LLP eSim setup = 4 partners + 1 compliance officer; laptop prompt fills tab 1 and stops on foreign ID type
From the QA's eSim LLP screenshot: partners are PT with Entity No. = LLP
number and ID Type 01 NRIC; keep one CO (Partner A, Entity No. blank);
never copy a block with a non-12-digit NRIC.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_015cZiRisoA6SpsRKpMC9zuJ
</commit_message>
<xml_diff>
--- a/EAINT-12341/cr/EAINT-12341/02-plan/EAINT-12341_eSim_Setup.xlsx
+++ b/EAINT-12341/cr/EAINT-12341/02-plan/EAINT-12341_eSim_Setup.xlsx
@@ -3699,7 +3699,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C39"/>
+  <dimension ref="A1:C46"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -3954,7 +3954,7 @@
     <row r="22">
       <c r="A22" s="10" t="inlineStr">
         <is>
-          <t>Part B — LLP is NOT in the eSimulator guide — send QA support a screenshot of one LLP record first</t>
+          <t>Part B — LLP record (from the QA's eSim screenshot, 02.10.2026)</t>
         </is>
       </c>
     </row>
@@ -3978,7 +3978,7 @@
     <row r="24">
       <c r="A24" s="6" t="inlineStr">
         <is>
-          <t>Registration number tag</t>
+          <t>LLP number</t>
         </is>
       </c>
       <c r="B24" s="8">
@@ -3987,89 +3987,89 @@
       </c>
       <c r="C24" s="6" t="inlineStr">
         <is>
-          <t>Whatever tag holds the LLP number — WITH '-LGN'</t>
+          <t>WITH '-LGN' — never split</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="6" t="inlineStr">
         <is>
-          <t>New number tag</t>
+          <t>New number</t>
         </is>
       </c>
       <c r="B25" s="8">
         <f>IF('1 Companies'!G9="","(fill tab 1 first)",'1 Companies'!G9)</f>
         <v/>
       </c>
-      <c r="C25" s="6" t="inlineStr"/>
-    </row>
-    <row r="26">
-      <c r="A26" s="6" t="inlineStr">
-        <is>
-          <t>Status tag</t>
-        </is>
-      </c>
-      <c r="B26" s="6" t="inlineStr">
-        <is>
-          <t>active / existing</t>
-        </is>
-      </c>
-      <c r="C26" s="6" t="inlineStr">
-        <is>
-          <t>Same idea as ROB / ROC — confirm on the screenshot</t>
+      <c r="C25" s="6" t="inlineStr">
+        <is>
+          <t>12 digits</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="10" t="inlineStr">
+        <is>
+          <t>Part B — 'Involvements': 4 PARTNER blocks + 1 COMPLIANCE OFFICER block</t>
         </is>
       </c>
     </row>
     <row r="28">
-      <c r="A28" s="10" t="inlineStr">
-        <is>
-          <t>Part B — text box 'Involvements': exactly 4 partner blocks (type PT, no compliance officer)</t>
+      <c r="A28" s="4" t="inlineStr">
+        <is>
+          <t>Field</t>
+        </is>
+      </c>
+      <c r="B28" s="4" t="inlineStr">
+        <is>
+          <t>Type this</t>
+        </is>
+      </c>
+      <c r="C28" s="4" t="inlineStr">
+        <is>
+          <t>Note</t>
         </is>
       </c>
     </row>
     <row r="29">
-      <c r="A29" s="4" t="inlineStr">
-        <is>
-          <t>Field</t>
-        </is>
-      </c>
-      <c r="B29" s="4" t="inlineStr">
-        <is>
-          <t>Type this</t>
-        </is>
-      </c>
-      <c r="C29" s="4" t="inlineStr">
-        <is>
-          <t>Note</t>
+      <c r="A29" s="6" t="inlineStr">
+        <is>
+          <t>Pattern</t>
+        </is>
+      </c>
+      <c r="B29" s="6" t="inlineStr">
+        <is>
+          <t>Copy an existing 'PT – Partner' block whose ID No. is a 12-digit NRIC</t>
+        </is>
+      </c>
+      <c r="C29" s="6" t="inlineStr">
+        <is>
+          <t>Do NOT copy a block whose ID No. is not 12 digits (e.g. RA0009999)</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="6" t="inlineStr">
         <is>
-          <t>Person A — name</t>
+          <t>Type (each partner)</t>
         </is>
       </c>
       <c r="B30" s="6" t="inlineStr">
         <is>
-          <t>QA DIRECTOR A</t>
-        </is>
-      </c>
-      <c r="C30" s="6" t="inlineStr">
-        <is>
-          <t>Malaysian</t>
-        </is>
-      </c>
+          <t>PT – Partner</t>
+        </is>
+      </c>
+      <c r="C30" s="6" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" s="6" t="inlineStr">
         <is>
-          <t>Person A — IC (no dashes)</t>
+          <t>ID Type (each partner)</t>
         </is>
       </c>
       <c r="B31" s="6" t="inlineStr">
         <is>
-          <t>690501137631</t>
+          <t>01 – NRIC</t>
         </is>
       </c>
       <c r="C31" s="6" t="inlineStr"/>
@@ -4077,29 +4077,28 @@
     <row r="32">
       <c r="A32" s="6" t="inlineStr">
         <is>
-          <t>Person B — name</t>
-        </is>
-      </c>
-      <c r="B32" s="6" t="inlineStr">
-        <is>
-          <t>QA DIRECTOR B</t>
-        </is>
+          <t>Entity No. (each partner)</t>
+        </is>
+      </c>
+      <c r="B32" s="8">
+        <f>IF('1 Companies'!F9="","(fill tab 1 first)",'1 Companies'!F9)</f>
+        <v/>
       </c>
       <c r="C32" s="6" t="inlineStr">
         <is>
-          <t>Malaysian</t>
+          <t>Your LLP number</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="6" t="inlineStr">
         <is>
-          <t>Person B — IC (no dashes)</t>
+          <t>Address / postcode / others</t>
         </is>
       </c>
       <c r="B33" s="6" t="inlineStr">
         <is>
-          <t>690502137632</t>
+          <t>leave as copied</t>
         </is>
       </c>
       <c r="C33" s="6" t="inlineStr"/>
@@ -4107,65 +4106,155 @@
     <row r="34">
       <c r="A34" s="6" t="inlineStr">
         <is>
-          <t>Person C — name</t>
+          <t>Compliance Officer block</t>
         </is>
       </c>
       <c r="B34" s="6" t="inlineStr">
         <is>
-          <t>QA DIRECTOR C</t>
+          <t>Type CO – Compliance Officer · ID Type 01 – NRIC · ID No. 690501137631 · Name QA DIRECTOR A · Entity No. blank</t>
         </is>
       </c>
       <c r="C34" s="6" t="inlineStr">
         <is>
-          <t>Malaysian</t>
+          <t>Same person as Partner A (as in the existing record). Keep exactly 1 CO.</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="6" t="inlineStr">
         <is>
-          <t>Person C — IC (no dashes)</t>
+          <t>Delete</t>
         </is>
       </c>
       <c r="B35" s="6" t="inlineStr">
         <is>
-          <t>690503137633</t>
+          <t>Any other partner / CO blocks from the copied record</t>
         </is>
       </c>
       <c r="C35" s="6" t="inlineStr"/>
-    </row>
-    <row r="36">
-      <c r="A36" s="6" t="inlineStr">
-        <is>
-          <t>Person D — name</t>
-        </is>
-      </c>
-      <c r="B36" s="6" t="inlineStr">
-        <is>
-          <t>QA DIRECTOR D</t>
-        </is>
-      </c>
-      <c r="C36" s="6" t="inlineStr">
-        <is>
-          <t>Malaysian</t>
-        </is>
-      </c>
     </row>
     <row r="37">
       <c r="A37" s="6" t="inlineStr">
         <is>
-          <t>Person D — IC (no dashes)</t>
+          <t>Person A — name</t>
         </is>
       </c>
       <c r="B37" s="6" t="inlineStr">
         <is>
+          <t>QA DIRECTOR A</t>
+        </is>
+      </c>
+      <c r="C37" s="6" t="inlineStr">
+        <is>
+          <t>Malaysian</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="6" t="inlineStr">
+        <is>
+          <t>Person A — ID No. (NRIC, no dashes)</t>
+        </is>
+      </c>
+      <c r="B38" s="6" t="inlineStr">
+        <is>
+          <t>690501137631</t>
+        </is>
+      </c>
+      <c r="C38" s="6" t="inlineStr"/>
+    </row>
+    <row r="39">
+      <c r="A39" s="6" t="inlineStr">
+        <is>
+          <t>Person B — name</t>
+        </is>
+      </c>
+      <c r="B39" s="6" t="inlineStr">
+        <is>
+          <t>QA DIRECTOR B</t>
+        </is>
+      </c>
+      <c r="C39" s="6" t="inlineStr">
+        <is>
+          <t>Malaysian</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="6" t="inlineStr">
+        <is>
+          <t>Person B — ID No. (NRIC, no dashes)</t>
+        </is>
+      </c>
+      <c r="B40" s="6" t="inlineStr">
+        <is>
+          <t>690502137632</t>
+        </is>
+      </c>
+      <c r="C40" s="6" t="inlineStr"/>
+    </row>
+    <row r="41">
+      <c r="A41" s="6" t="inlineStr">
+        <is>
+          <t>Person C — name</t>
+        </is>
+      </c>
+      <c r="B41" s="6" t="inlineStr">
+        <is>
+          <t>QA DIRECTOR C</t>
+        </is>
+      </c>
+      <c r="C41" s="6" t="inlineStr">
+        <is>
+          <t>Malaysian</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="6" t="inlineStr">
+        <is>
+          <t>Person C — ID No. (NRIC, no dashes)</t>
+        </is>
+      </c>
+      <c r="B42" s="6" t="inlineStr">
+        <is>
+          <t>690503137633</t>
+        </is>
+      </c>
+      <c r="C42" s="6" t="inlineStr"/>
+    </row>
+    <row r="43">
+      <c r="A43" s="6" t="inlineStr">
+        <is>
+          <t>Person D — name</t>
+        </is>
+      </c>
+      <c r="B43" s="6" t="inlineStr">
+        <is>
+          <t>QA DIRECTOR D</t>
+        </is>
+      </c>
+      <c r="C43" s="6" t="inlineStr">
+        <is>
+          <t>Malaysian</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="6" t="inlineStr">
+        <is>
+          <t>Person D — ID No. (NRIC, no dashes)</t>
+        </is>
+      </c>
+      <c r="B44" s="6" t="inlineStr">
+        <is>
           <t>690504137634</t>
         </is>
       </c>
-      <c r="C37" s="6" t="inlineStr"/>
-    </row>
-    <row r="39">
-      <c r="A39" s="3" t="inlineStr">
+      <c r="C44" s="6" t="inlineStr"/>
+    </row>
+    <row r="46">
+      <c r="A46" s="3" t="inlineStr">
         <is>
           <t>Then: Save, tell QA support 'eSim ready', and run the robot.</t>
         </is>
@@ -4173,8 +4262,8 @@
     </row>
   </sheetData>
   <mergeCells count="4">
-    <mergeCell ref="A28:C28"/>
     <mergeCell ref="A4:C4"/>
+    <mergeCell ref="A27:C27"/>
     <mergeCell ref="A13:C13"/>
     <mergeCell ref="A22:C22"/>
   </mergeCells>

</xml_diff>